<commit_message>
1.3.1- Testing Signup functionality by giving Valid credentials
</commit_message>
<xml_diff>
--- a/Facebook-Automation-Test/src/Test Cases.xlsx
+++ b/Facebook-Automation-Test/src/Test Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\QA\My QA Projects\Facebook Automation Test\Facebook-Automation-Test\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8ED890A3-6A0A-46E0-8CF1-45089E8DDAE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AEE8B57-A851-4433-9DAE-F3B5805C914E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="0" windowWidth="23256" windowHeight="7488" xr2:uid="{560DE587-4291-4869-85E5-DA09B090168E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{560DE587-4291-4869-85E5-DA09B090168E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="87">
   <si>
     <t>Project Name</t>
   </si>
@@ -160,21 +160,11 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Username - aaabbb@gmail.com
-Password - Celkon
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Username - jigiwi7156@jofuso.com
 Password - xxxx
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Username - aaabbb@gmail.com
-Password - xxxx
-</t>
-  </si>
-  <si>
     <t>User should be able to see Facebook Home Page</t>
   </si>
   <si>
@@ -186,6 +176,206 @@
   <si>
     <t>Sometimes while Anonymous 
 Login it is requiring the password again</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error Message </t>
+  </si>
+  <si>
+    <t>Show error message "invalid Username /  Password"</t>
+  </si>
+  <si>
+    <t>Error Message is
+Showing sometimes only</t>
+  </si>
+  <si>
+    <t>Showing error message "invalid Username /  Password"</t>
+  </si>
+  <si>
+    <t>Functioning
+Successful Login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Username -fefah24039@eoilup.com
+Password - Celkon
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Username - fefah24039@eoilup.com
+Password - Micromax
+</t>
+  </si>
+  <si>
+    <t>Signup</t>
+  </si>
+  <si>
+    <t>13/10/2024</t>
+  </si>
+  <si>
+    <t>TS_FB_02</t>
+  </si>
+  <si>
+    <t>Verify Login Fucntionality of 
+FaceBook Signup page</t>
+  </si>
+  <si>
+    <t>TC_FB_Signup_01</t>
+  </si>
+  <si>
+    <t>TC_FB_Signup_02</t>
+  </si>
+  <si>
+    <t>TC_FB_Signup_03</t>
+  </si>
+  <si>
+    <t>TC_FB_Signup_04</t>
+  </si>
+  <si>
+    <t>TC_FB_Signup_05</t>
+  </si>
+  <si>
+    <t>TC_FB_Signup_06</t>
+  </si>
+  <si>
+    <t>Enter valid name, valid birthdate, valid gender, valid email and invalid password</t>
+  </si>
+  <si>
+    <t>TC_FB_Signup_07</t>
+  </si>
+  <si>
+    <t>TC_FB_Signup_08</t>
+  </si>
+  <si>
+    <t>01. Enter a valid name 
+02. Enter a valid Birthdate
+03. Check gender is Selected
+04. Enter a invalid email
+05. Enter a valid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>Enter valid name, valid birthdate, Check gender is Selected, valid email and valid password</t>
+  </si>
+  <si>
+    <t>Enter invalid name, valid birthdate, Check gender is Selected, valid email and valid password</t>
+  </si>
+  <si>
+    <t>Enter valid name, invalid birthdateCheck gender is Selected, valid email and valid password</t>
+  </si>
+  <si>
+    <t>Enter valid name, invalid birthdate, Check gender is Selected, invalid email and valid password</t>
+  </si>
+  <si>
+    <t>Don't enter name, Enter valid birthdate, Check gender is Selected, valid email, valid password</t>
+  </si>
+  <si>
+    <t>Enter valid name, valid birthdate, Check gender is Selected, Don't enter email ,Enter valid password</t>
+  </si>
+  <si>
+    <t>valid name, valid birthdate, Check gender is Selected, valid email, Don't enter password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Name - Kavishka
+Surname - Rathnayaka
+Birthdate - 27/Jan/2001
+Email - 
+Password - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Name - 4
+Surname - 6
+Birthdate - 27/Jan/2001
+Email - 
+Password - </t>
+  </si>
+  <si>
+    <t>Error Message</t>
+  </si>
+  <si>
+    <t>Successful Account Creation</t>
+  </si>
+  <si>
+    <t>First Name - Kavishka
+Surname - Rathnayaka
+Birthdate - 27/Jan/2001
+Email - 
+Password - xxxx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Name - 
+Surname - 
+Birthdate - 27/Jan/2001
+Email - 
+Password - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Name - Kavishka
+Surname - Rathnayaka
+Birthdate - 01/Apr/2024
+Email - 
+Password - </t>
+  </si>
+  <si>
+    <t>01. Don't enter name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter Male
+04. Enter a valid email
+05. Enter a valid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>01. Enter a valid name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter Male
+04. Don't enter email
+05. Enter a valid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>01. Enter a valid name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter Male
+04. Enter a valid email
+05. Don't enter password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>01. Enter a valid name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter FeMale
+04. Enter a valid email
+05. Enter a invalid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>01. Enter a invalid name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter Female
+04. Enter a valid email
+05. Enter a valid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>01. Enter a valid name 
+02. Enter a invalid Birthdate
+03. Check gender is Selected/Enter Custom
+04. Enter a valid email
+05. Enter a valid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>01. Enter a valid name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter Female
+04. Enter a valid email
+05. Enter a valid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>First Name - Kaveesha
+Surname - Rathnayaka
+Birthdate - 27/Jan/2001
+Email - fefah24039@eoilup.com
+Password - Celkon</t>
   </si>
 </sst>
 </file>
@@ -239,31 +429,82 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+  <dxfs count="32">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -286,6 +527,72 @@
       </fill>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -300,23 +607,46 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B9F8EB46-DB7B-47C8-95C7-454F508025A7}" name="Table4" displayName="Table4" ref="A8:N12" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B9F8EB46-DB7B-47C8-95C7-454F508025A7}" name="Table4" displayName="Table4" ref="A8:N12" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
   <autoFilter ref="A8:N12" xr:uid="{B9F8EB46-DB7B-47C8-95C7-454F508025A7}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{FA1520E5-151F-4C35-9564-490E6E227E63}" name="Test Scenario ID"/>
-    <tableColumn id="2" xr3:uid="{4CD9CF72-D3D5-4E13-B21F-2628B71CA730}" name="Test Scenario Description"/>
-    <tableColumn id="3" xr3:uid="{64C682F3-74F4-4B58-9AAA-079E2202EC63}" name="Test Case ID"/>
-    <tableColumn id="4" xr3:uid="{F8711D9F-D3E9-4C0E-83A5-1112EACF3ECF}" name="Test Case Description"/>
-    <tableColumn id="5" xr3:uid="{3C9E830E-1C51-4CB9-9B33-8A5AFEEE698E}" name="Test Steps"/>
-    <tableColumn id="13" xr3:uid="{795BF8D4-2BAA-4AD4-842A-88C791483F7A}" name="Preconditions" dataDxfId="2"/>
-    <tableColumn id="14" xr3:uid="{21B04C03-953D-42FE-8068-4BF43AFF3291}" name="Test Data" dataDxfId="1"/>
-    <tableColumn id="15" xr3:uid="{9CF2DA71-3D28-4A14-A4CE-044972166E7C}" name="Post conditions" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{42C30692-F71E-4898-A159-20BE875D8033}" name="Expected Result"/>
-    <tableColumn id="7" xr3:uid="{03D56321-2D40-4418-8D06-EED641A4F370}" name="Actual Result"/>
-    <tableColumn id="8" xr3:uid="{C0EAC999-BB87-4D0C-9360-9BFF9AF67768}" name="Status"/>
-    <tableColumn id="9" xr3:uid="{3B92054E-DFF9-4A75-AF0B-7B5080A92062}" name="Executed by"/>
-    <tableColumn id="10" xr3:uid="{E7860CF1-1E6C-471A-B8FB-6DB223239798}" name="Executed Date"/>
-    <tableColumn id="11" xr3:uid="{D4382055-B4B2-40BA-B30A-2EE9840623E1}" name="Comments (Any)"/>
+    <tableColumn id="1" xr3:uid="{FA1520E5-151F-4C35-9564-490E6E227E63}" name="Test Scenario ID" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{4CD9CF72-D3D5-4E13-B21F-2628B71CA730}" name="Test Scenario Description" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{64C682F3-74F4-4B58-9AAA-079E2202EC63}" name="Test Case ID" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{F8711D9F-D3E9-4C0E-83A5-1112EACF3ECF}" name="Test Case Description" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{3C9E830E-1C51-4CB9-9B33-8A5AFEEE698E}" name="Test Steps" dataDxfId="25"/>
+    <tableColumn id="13" xr3:uid="{795BF8D4-2BAA-4AD4-842A-88C791483F7A}" name="Preconditions" dataDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{21B04C03-953D-42FE-8068-4BF43AFF3291}" name="Test Data" dataDxfId="23"/>
+    <tableColumn id="15" xr3:uid="{9CF2DA71-3D28-4A14-A4CE-044972166E7C}" name="Post conditions" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{42C30692-F71E-4898-A159-20BE875D8033}" name="Expected Result" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{03D56321-2D40-4418-8D06-EED641A4F370}" name="Actual Result" dataDxfId="20"/>
+    <tableColumn id="8" xr3:uid="{C0EAC999-BB87-4D0C-9360-9BFF9AF67768}" name="Status" dataDxfId="19"/>
+    <tableColumn id="9" xr3:uid="{3B92054E-DFF9-4A75-AF0B-7B5080A92062}" name="Executed by" dataDxfId="18"/>
+    <tableColumn id="10" xr3:uid="{E7860CF1-1E6C-471A-B8FB-6DB223239798}" name="Executed Date" dataDxfId="17"/>
+    <tableColumn id="11" xr3:uid="{D4382055-B4B2-40BA-B30A-2EE9840623E1}" name="Comments (Any)" dataDxfId="16"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B1155A5B-1493-4085-854F-C5DA20AD28C9}" name="Table42" displayName="Table42" ref="A23:N31" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+  <autoFilter ref="A23:N31" xr:uid="{B1155A5B-1493-4085-854F-C5DA20AD28C9}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{B343AAFA-6457-4739-9100-101EF218F54D}" name="Test Scenario ID" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{E5529356-E16E-4EC4-9C43-4E830FC2E50F}" name="Test Scenario Description" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{2551A72A-8D4F-449F-B940-710504664FA5}" name="Test Case ID" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{00ECB93F-754B-43F5-9E43-F3D6BB21402C}" name="Test Case Description" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{66E4AAFF-0A66-44A2-A53B-7FABEAD85F8D}" name="Test Steps" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{662ABFF6-2773-475F-B091-BCDABF3FB4DE}" name="Preconditions" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{671E1D04-8126-4597-BD89-AC9A178AC6EA}" name="Test Data" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{90971945-FDC9-429A-8527-A13B23E811A8}" name="Post conditions" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{EF04FFC6-AA15-47C8-B4A9-828B2777CD1D}" name="Expected Result" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{4CA89147-B985-4D56-876B-62F63DC92C49}" name="Actual Result" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{BDA4C2F1-0AF2-488C-953C-82660F211B43}" name="Status" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{EF661887-7461-490A-8D26-42708C7DEF3D}" name="Executed by" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{BD8FCAC9-00C9-4F76-A5CA-C0CB2DE0CB76}" name="Executed Date" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{C33D96A1-29CA-4A83-BFA6-64CF06278883}" name="Comments (Any)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -619,27 +949,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32799D75-E317-4EA9-991F-FF31DA4317A3}">
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
     <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" customWidth="1"/>
     <col min="4" max="4" width="20.5546875" customWidth="1"/>
-    <col min="5" max="5" width="24.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.6640625" customWidth="1"/>
     <col min="6" max="6" width="16.5546875" customWidth="1"/>
     <col min="7" max="7" width="21.109375" customWidth="1"/>
     <col min="8" max="8" width="14.88671875" customWidth="1"/>
     <col min="9" max="9" width="16.77734375" customWidth="1"/>
-    <col min="10" max="10" width="14.88671875" customWidth="1"/>
+    <col min="10" max="10" width="17.21875" customWidth="1"/>
     <col min="11" max="11" width="10.88671875" customWidth="1"/>
-    <col min="12" max="12" width="14.33203125" customWidth="1"/>
+    <col min="12" max="12" width="18.33203125" customWidth="1"/>
     <col min="13" max="13" width="15" customWidth="1"/>
     <col min="14" max="14" width="27.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -647,7 +977,7 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
@@ -655,7 +985,7 @@
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
@@ -663,7 +993,7 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1">
@@ -671,156 +1001,638 @@
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="B6" s="1">
+        <v>45636</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="L8" s="4" t="s">
+      <c r="L8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="N8" s="4" t="s">
+      <c r="N8" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K9" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I9" t="s">
+      <c r="L9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M9" s="7">
+        <v>45636</v>
+      </c>
+      <c r="N9" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="J9" t="s">
-        <v>43</v>
-      </c>
-      <c r="K9" t="s">
+    </row>
+    <row r="10" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="I10" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="J10" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M10" s="7">
+        <v>45636</v>
+      </c>
+      <c r="N10" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M11" s="7">
+        <v>45636</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M12" s="7">
+        <v>45636</v>
+      </c>
+      <c r="N12" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="1">
+        <v>45636</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="N23" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="H24" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" s="2" t="s">
+      <c r="I24" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="N24" s="5"/>
+    </row>
+    <row r="25" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F25" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="C12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="G25" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M25" s="7">
+        <v>45636</v>
+      </c>
+      <c r="N25" s="5"/>
+    </row>
+    <row r="26" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F26" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H12" s="2"/>
-    </row>
+      <c r="G26" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M26" s="7">
+        <v>45636</v>
+      </c>
+      <c r="N26" s="5"/>
+    </row>
+    <row r="27" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M27" s="7"/>
+      <c r="N27" s="5"/>
+    </row>
+    <row r="28" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M28" s="7"/>
+      <c r="N28" s="5"/>
+    </row>
+    <row r="29" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L29" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M29" s="7"/>
+      <c r="N29" s="5"/>
+    </row>
+    <row r="30" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L30" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M30" s="7"/>
+      <c r="N30" s="5"/>
+    </row>
+    <row r="31" spans="1:14" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H31" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L31" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M31" s="7"/>
+      <c r="N31" s="5"/>
+    </row>
+    <row r="32" spans="1:14" ht="87" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1.3.2- Testing Signup functionality by giving invalid Birthdate and valid data
</commit_message>
<xml_diff>
--- a/Facebook-Automation-Test/src/Test Cases.xlsx
+++ b/Facebook-Automation-Test/src/Test Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\QA\My QA Projects\Facebook Automation Test\Facebook-Automation-Test\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AEE8B57-A851-4433-9DAE-F3B5805C914E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13911504-2EF9-4B8D-B73A-09761E8AEBAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{560DE587-4291-4869-85E5-DA09B090168E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="90">
   <si>
     <t>Project Name</t>
   </si>
@@ -206,9 +206,6 @@
   </si>
   <si>
     <t>Signup</t>
-  </si>
-  <si>
-    <t>13/10/2024</t>
   </si>
   <si>
     <t>TS_FB_02</t>
@@ -281,13 +278,6 @@
 Password - </t>
   </si>
   <si>
-    <t xml:space="preserve">First Name - 4
-Surname - 6
-Birthdate - 27/Jan/2001
-Email - 
-Password - </t>
-  </si>
-  <si>
     <t>Error Message</t>
   </si>
   <si>
@@ -304,13 +294,6 @@
     <t xml:space="preserve">First Name - 
 Surname - 
 Birthdate - 27/Jan/2001
-Email - 
-Password - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">First Name - Kavishka
-Surname - Rathnayaka
-Birthdate - 01/Apr/2024
 Email - 
 Password - </t>
   </si>
@@ -347,14 +330,6 @@
 06. Click on Signup Button</t>
   </si>
   <si>
-    <t>01. Enter a invalid name 
-02. Enter a valid Birthdate
-03. Check gender is Selected/Enter Female
-04. Enter a valid email
-05. Enter a valid password
-06. Click on Signup Button</t>
-  </si>
-  <si>
     <t>01. Enter a valid name 
 02. Enter a invalid Birthdate
 03. Check gender is Selected/Enter Custom
@@ -376,6 +351,40 @@
 Birthdate - 27/Jan/2001
 Email - fefah24039@eoilup.com
 Password - Celkon</t>
+  </si>
+  <si>
+    <t>Show error message "This name contains certain characters that aren't allowed"</t>
+  </si>
+  <si>
+    <t>01. Enter an invalid name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter male
+04. Enter a valid email
+05. Enter a valid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>First Name - 4
+Surname - 6
+Birthdate - 27/Jan/2001
+Email - fefah24039@eoilup.com
+Password - Celkon</t>
+  </si>
+  <si>
+    <t>First Name - Medhanga
+Surname - Bandara
+Birthdate - 01/Apr/2024
+Email - fefah24039@eoilup.com
+Password - Celkon</t>
+  </si>
+  <si>
+    <t>Show error message "It looks like you've entered the wrong info. Please make sure that you use your real date of birth"</t>
+  </si>
+  <si>
+    <t>Showing error message "This name contains certain characters that aren't allowed"</t>
+  </si>
+  <si>
+    <t>Showing error message "It looks like you've entered the wrong info. Please make sure that you use your real date of birth"</t>
   </si>
 </sst>
 </file>
@@ -1264,8 +1273,8 @@
       <c r="A19" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>52</v>
+      <c r="B19" s="1">
+        <v>45637</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
@@ -1330,34 +1339,34 @@
     </row>
     <row r="24" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>55</v>
-      </c>
       <c r="D24" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>40</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K24" s="6" t="s">
         <v>42</v>
@@ -1365,38 +1374,42 @@
       <c r="L24" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="M24" s="7" t="s">
-        <v>52</v>
+      <c r="M24" s="7">
+        <v>45637</v>
       </c>
       <c r="N24" s="5"/>
     </row>
     <row r="25" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="C25" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
+        <v>72</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="K25" s="6" t="s">
         <v>42</v>
       </c>
@@ -1404,37 +1417,41 @@
         <v>32</v>
       </c>
       <c r="M25" s="7">
-        <v>45636</v>
+        <v>45637</v>
       </c>
       <c r="N25" s="5"/>
     </row>
-    <row r="26" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" ht="115.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="C26" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
+        <v>72</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>89</v>
+      </c>
       <c r="K26" s="6" t="s">
         <v>42</v>
       </c>
@@ -1442,34 +1459,34 @@
         <v>32</v>
       </c>
       <c r="M26" s="7">
-        <v>45636</v>
+        <v>45637</v>
       </c>
       <c r="N26" s="5"/>
     </row>
     <row r="27" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="C27" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F27" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G27" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H27" s="8" t="s">
         <v>72</v>
-      </c>
-      <c r="H27" s="8" t="s">
-        <v>74</v>
       </c>
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
@@ -1484,28 +1501,28 @@
     </row>
     <row r="28" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="C28" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
@@ -1520,28 +1537,28 @@
     </row>
     <row r="29" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="C29" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F29" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
@@ -1556,28 +1573,28 @@
     </row>
     <row r="30" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="C30" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F30" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G30" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H30" s="8" t="s">
         <v>72</v>
-      </c>
-      <c r="H30" s="8" t="s">
-        <v>74</v>
       </c>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
@@ -1592,28 +1609,28 @@
     </row>
     <row r="31" spans="1:14" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="C31" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F31" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G31" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H31" s="8" t="s">
         <v>72</v>
-      </c>
-      <c r="H31" s="8" t="s">
-        <v>74</v>
       </c>
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>

</xml_diff>

<commit_message>
Test Cases of the Project
</commit_message>
<xml_diff>
--- a/Facebook-Automation-Test/src/Test Cases.xlsx
+++ b/Facebook-Automation-Test/src/Test Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\QA\My QA Projects\Facebook Automation Test\Facebook-Automation-Test\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13911504-2EF9-4B8D-B73A-09761E8AEBAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12013B6A-B1E1-4B57-9643-026F2CF00995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{560DE587-4291-4869-85E5-DA09B090168E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="102">
   <si>
     <t>Project Name</t>
   </si>
@@ -169,9 +169,6 @@
   </si>
   <si>
     <t>Successful Login</t>
-  </si>
-  <si>
-    <t>Passed</t>
   </si>
   <si>
     <t>Sometimes while Anonymous 
@@ -271,39 +268,10 @@
     <t>valid name, valid birthdate, Check gender is Selected, valid email, Don't enter password</t>
   </si>
   <si>
-    <t xml:space="preserve">First Name - Kavishka
-Surname - Rathnayaka
-Birthdate - 27/Jan/2001
-Email - 
-Password - </t>
-  </si>
-  <si>
     <t>Error Message</t>
   </si>
   <si>
     <t>Successful Account Creation</t>
-  </si>
-  <si>
-    <t>First Name - Kavishka
-Surname - Rathnayaka
-Birthdate - 27/Jan/2001
-Email - 
-Password - xxxx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First Name - 
-Surname - 
-Birthdate - 27/Jan/2001
-Email - 
-Password - </t>
-  </si>
-  <si>
-    <t>01. Don't enter name 
-02. Enter a valid Birthdate
-03. Check gender is Selected/Enter Male
-04. Enter a valid email
-05. Enter a valid password
-06. Click on Signup Button</t>
   </si>
   <si>
     <t>01. Enter a valid name 
@@ -315,22 +283,6 @@
   </si>
   <si>
     <t>01. Enter a valid name 
-02. Enter a valid Birthdate
-03. Check gender is Selected/Enter Male
-04. Enter a valid email
-05. Don't enter password
-06. Click on Signup Button</t>
-  </si>
-  <si>
-    <t>01. Enter a valid name 
-02. Enter a valid Birthdate
-03. Check gender is Selected/Enter FeMale
-04. Enter a valid email
-05. Enter a invalid password
-06. Click on Signup Button</t>
-  </si>
-  <si>
-    <t>01. Enter a valid name 
 02. Enter a invalid Birthdate
 03. Check gender is Selected/Enter Custom
 04. Enter a valid email
@@ -385,6 +337,98 @@
   </si>
   <si>
     <t>Showing error message "It looks like you've entered the wrong info. Please make sure that you use your real date of birth"</t>
+  </si>
+  <si>
+    <t>Show error message "Please enter a valid mobile number or email address."</t>
+  </si>
+  <si>
+    <t>Showing error message "Please enter a valid mobile number or email address."</t>
+  </si>
+  <si>
+    <t>First Name - Kavishka
+Surname - Rathnayaka
+Birthdate - 27/Jan/2001
+Email - hovihama.lk
+Password - Celkon</t>
+  </si>
+  <si>
+    <t>First Name - Kaveesha
+Surname - Rathnayaka
+Birthdate - 27/Jan/2001
+Email - fefah24039@eoilup.com
+Password - xxxx</t>
+  </si>
+  <si>
+    <t>Show error message "Your password must be at least 6 characters long. Please try another."</t>
+  </si>
+  <si>
+    <t>Showing error message "Your password must be at least 6 characters long. Please try another."</t>
+  </si>
+  <si>
+    <t>Show error message "What's your name?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Name - 
+Surname - 
+Birthdate - 27/Jan/2001
+Email - fefah24039@eoilup.com
+Password - Celkon </t>
+  </si>
+  <si>
+    <t>Show error message "You'll use this when you log in and if you ever need to reset your password."</t>
+  </si>
+  <si>
+    <t>Showing error message "You'll use this when you log in and if you ever need to reset your password."</t>
+  </si>
+  <si>
+    <t>Showing error message "What's your name?"</t>
+  </si>
+  <si>
+    <t>Show error message "Enter a combination of at least six numbers, letters and punctuation marks."</t>
+  </si>
+  <si>
+    <t>Showing error message "Enter a combination of at least six numbers, letters and punctuation marks."</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>First Name - Kaveesha
+Surname - Rathnayaka
+Birthdate - 27/Jan/2001
+Email - 
+Password - Celkon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Name - Kaveesha
+Surname - Rathnayaka
+Birthdate - 27/Jan/2001
+Email - fefah24039@eoilup.com
+Password - </t>
+  </si>
+  <si>
+    <t>01. Don't enter name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter Female
+04. Enter a valid email
+05. Enter a valid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>01. Enter a valid name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter Female
+04. Enter a valid email
+05. Enter a invalid password
+06. Click on Signup Button</t>
+  </si>
+  <si>
+    <t>01. Enter a valid name 
+02. Enter a valid Birthdate
+03. Check gender is Selected/Enter Female
+04. Enter a valid email
+05. Don't enter password
+06. Click on Signup Button</t>
   </si>
 </sst>
 </file>
@@ -412,7 +456,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -422,6 +466,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -438,7 +488,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -465,6 +515,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,51 +591,6 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -597,10 +606,55 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.59999389629810485"/>
+          <bgColor theme="9" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -616,46 +670,46 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B9F8EB46-DB7B-47C8-95C7-454F508025A7}" name="Table4" displayName="Table4" ref="A8:N12" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B9F8EB46-DB7B-47C8-95C7-454F508025A7}" name="Table4" displayName="Table4" ref="A8:N12" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A8:N12" xr:uid="{B9F8EB46-DB7B-47C8-95C7-454F508025A7}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{FA1520E5-151F-4C35-9564-490E6E227E63}" name="Test Scenario ID" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{4CD9CF72-D3D5-4E13-B21F-2628B71CA730}" name="Test Scenario Description" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{64C682F3-74F4-4B58-9AAA-079E2202EC63}" name="Test Case ID" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{F8711D9F-D3E9-4C0E-83A5-1112EACF3ECF}" name="Test Case Description" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{3C9E830E-1C51-4CB9-9B33-8A5AFEEE698E}" name="Test Steps" dataDxfId="25"/>
-    <tableColumn id="13" xr3:uid="{795BF8D4-2BAA-4AD4-842A-88C791483F7A}" name="Preconditions" dataDxfId="24"/>
-    <tableColumn id="14" xr3:uid="{21B04C03-953D-42FE-8068-4BF43AFF3291}" name="Test Data" dataDxfId="23"/>
-    <tableColumn id="15" xr3:uid="{9CF2DA71-3D28-4A14-A4CE-044972166E7C}" name="Post conditions" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{42C30692-F71E-4898-A159-20BE875D8033}" name="Expected Result" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{03D56321-2D40-4418-8D06-EED641A4F370}" name="Actual Result" dataDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{C0EAC999-BB87-4D0C-9360-9BFF9AF67768}" name="Status" dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{3B92054E-DFF9-4A75-AF0B-7B5080A92062}" name="Executed by" dataDxfId="18"/>
-    <tableColumn id="10" xr3:uid="{E7860CF1-1E6C-471A-B8FB-6DB223239798}" name="Executed Date" dataDxfId="17"/>
-    <tableColumn id="11" xr3:uid="{D4382055-B4B2-40BA-B30A-2EE9840623E1}" name="Comments (Any)" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{FA1520E5-151F-4C35-9564-490E6E227E63}" name="Test Scenario ID" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{4CD9CF72-D3D5-4E13-B21F-2628B71CA730}" name="Test Scenario Description" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{64C682F3-74F4-4B58-9AAA-079E2202EC63}" name="Test Case ID" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{F8711D9F-D3E9-4C0E-83A5-1112EACF3ECF}" name="Test Case Description" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{3C9E830E-1C51-4CB9-9B33-8A5AFEEE698E}" name="Test Steps" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{795BF8D4-2BAA-4AD4-842A-88C791483F7A}" name="Preconditions" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{21B04C03-953D-42FE-8068-4BF43AFF3291}" name="Test Data" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{9CF2DA71-3D28-4A14-A4CE-044972166E7C}" name="Post conditions" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{42C30692-F71E-4898-A159-20BE875D8033}" name="Expected Result" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{03D56321-2D40-4418-8D06-EED641A4F370}" name="Actual Result" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{C0EAC999-BB87-4D0C-9360-9BFF9AF67768}" name="Status" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{3B92054E-DFF9-4A75-AF0B-7B5080A92062}" name="Executed by" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{E7860CF1-1E6C-471A-B8FB-6DB223239798}" name="Executed Date" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{D4382055-B4B2-40BA-B30A-2EE9840623E1}" name="Comments (Any)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B1155A5B-1493-4085-854F-C5DA20AD28C9}" name="Table42" displayName="Table42" ref="A23:N31" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B1155A5B-1493-4085-854F-C5DA20AD28C9}" name="Table42" displayName="Table42" ref="A23:N31" totalsRowShown="0" headerRowDxfId="16" dataDxfId="31">
   <autoFilter ref="A23:N31" xr:uid="{B1155A5B-1493-4085-854F-C5DA20AD28C9}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{B343AAFA-6457-4739-9100-101EF218F54D}" name="Test Scenario ID" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{E5529356-E16E-4EC4-9C43-4E830FC2E50F}" name="Test Scenario Description" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{2551A72A-8D4F-449F-B940-710504664FA5}" name="Test Case ID" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{00ECB93F-754B-43F5-9E43-F3D6BB21402C}" name="Test Case Description" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{66E4AAFF-0A66-44A2-A53B-7FABEAD85F8D}" name="Test Steps" dataDxfId="9"/>
-    <tableColumn id="13" xr3:uid="{662ABFF6-2773-475F-B091-BCDABF3FB4DE}" name="Preconditions" dataDxfId="8"/>
-    <tableColumn id="14" xr3:uid="{671E1D04-8126-4597-BD89-AC9A178AC6EA}" name="Test Data" dataDxfId="7"/>
-    <tableColumn id="15" xr3:uid="{90971945-FDC9-429A-8527-A13B23E811A8}" name="Post conditions" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{EF04FFC6-AA15-47C8-B4A9-828B2777CD1D}" name="Expected Result" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{4CA89147-B985-4D56-876B-62F63DC92C49}" name="Actual Result" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{BDA4C2F1-0AF2-488C-953C-82660F211B43}" name="Status" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{EF661887-7461-490A-8D26-42708C7DEF3D}" name="Executed by" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{BD8FCAC9-00C9-4F76-A5CA-C0CB2DE0CB76}" name="Executed Date" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{C33D96A1-29CA-4A83-BFA6-64CF06278883}" name="Comments (Any)" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{B343AAFA-6457-4739-9100-101EF218F54D}" name="Test Scenario ID" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{E5529356-E16E-4EC4-9C43-4E830FC2E50F}" name="Test Scenario Description" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{2551A72A-8D4F-449F-B940-710504664FA5}" name="Test Case ID" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{00ECB93F-754B-43F5-9E43-F3D6BB21402C}" name="Test Case Description" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{66E4AAFF-0A66-44A2-A53B-7FABEAD85F8D}" name="Test Steps" dataDxfId="26"/>
+    <tableColumn id="13" xr3:uid="{662ABFF6-2773-475F-B091-BCDABF3FB4DE}" name="Preconditions" dataDxfId="25"/>
+    <tableColumn id="14" xr3:uid="{671E1D04-8126-4597-BD89-AC9A178AC6EA}" name="Test Data" dataDxfId="24"/>
+    <tableColumn id="15" xr3:uid="{90971945-FDC9-429A-8527-A13B23E811A8}" name="Post conditions" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{EF04FFC6-AA15-47C8-B4A9-828B2777CD1D}" name="Expected Result" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{4CA89147-B985-4D56-876B-62F63DC92C49}" name="Actual Result" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{BDA4C2F1-0AF2-488C-953C-82660F211B43}" name="Status" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{EF661887-7461-490A-8D26-42708C7DEF3D}" name="Executed by" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{BD8FCAC9-00C9-4F76-A5CA-C0CB2DE0CB76}" name="Executed Date" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{C33D96A1-29CA-4A83-BFA6-64CF06278883}" name="Comments (Any)" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -969,8 +1023,7 @@
     <col min="6" max="6" width="16.5546875" customWidth="1"/>
     <col min="7" max="7" width="21.109375" customWidth="1"/>
     <col min="8" max="8" width="14.88671875" customWidth="1"/>
-    <col min="9" max="9" width="16.77734375" customWidth="1"/>
-    <col min="10" max="10" width="17.21875" customWidth="1"/>
+    <col min="9" max="10" width="17.21875" customWidth="1"/>
     <col min="11" max="11" width="10.88671875" customWidth="1"/>
     <col min="12" max="12" width="18.33203125" customWidth="1"/>
     <col min="13" max="13" width="15" customWidth="1"/>
@@ -1098,10 +1151,10 @@
         <v>41</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L9" s="4" t="s">
         <v>32</v>
@@ -1110,7 +1163,7 @@
         <v>45636</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
@@ -1136,16 +1189,16 @@
         <v>39</v>
       </c>
       <c r="H10" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I10" s="5" t="s">
-        <v>45</v>
-      </c>
       <c r="J10" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L10" s="4" t="s">
         <v>32</v>
@@ -1154,7 +1207,7 @@
         <v>45636</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="72" x14ac:dyDescent="0.3">
@@ -1177,19 +1230,19 @@
         <v>33</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H11" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I11" s="5" t="s">
-        <v>45</v>
-      </c>
       <c r="J11" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L11" s="4" t="s">
         <v>32</v>
@@ -1198,7 +1251,7 @@
         <v>45636</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="72" x14ac:dyDescent="0.3">
@@ -1221,19 +1274,19 @@
         <v>33</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H12" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I12" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I12" s="5" t="s">
-        <v>45</v>
-      </c>
       <c r="J12" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L12" s="4" t="s">
         <v>32</v>
@@ -1242,11 +1295,11 @@
         <v>45636</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B16" t="s">
@@ -1254,15 +1307,15 @@
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="10" t="s">
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="10" t="s">
         <v>2</v>
       </c>
       <c r="B18" t="s">
@@ -1270,7 +1323,7 @@
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B19" s="1">
@@ -1278,7 +1331,7 @@
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="10" t="s">
         <v>4</v>
       </c>
       <c r="B20" t="s">
@@ -1286,90 +1339,90 @@
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="10" t="s">
         <v>5</v>
       </c>
       <c r="B21" s="1">
-        <v>45636</v>
+        <v>45639</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G23" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H23" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="I23" s="3" t="s">
+      <c r="I23" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="J23" s="3" t="s">
+      <c r="J23" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="K23" s="3" t="s">
+      <c r="K23" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="L23" s="3" t="s">
+      <c r="L23" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="M23" s="3" t="s">
+      <c r="M23" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="N23" s="3" t="s">
+      <c r="N23" s="11" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>54</v>
-      </c>
       <c r="D24" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>40</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L24" s="4" t="s">
         <v>32</v>
@@ -1381,37 +1434,37 @@
     </row>
     <row r="25" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="C25" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L25" s="4" t="s">
         <v>32</v>
@@ -1423,37 +1476,37 @@
     </row>
     <row r="26" spans="1:14" ht="115.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="C26" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L26" s="4" t="s">
         <v>32</v>
@@ -1463,187 +1516,217 @@
       </c>
       <c r="N26" s="5"/>
     </row>
-    <row r="27" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" ht="111.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="C27" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F27" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
+        <v>70</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="K27" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L27" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="M27" s="7"/>
+      <c r="M27" s="7">
+        <v>45638</v>
+      </c>
       <c r="N27" s="5"/>
     </row>
     <row r="28" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="C28" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
+        <v>70</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="K28" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L28" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="M28" s="7"/>
+      <c r="M28" s="7">
+        <v>45638</v>
+      </c>
       <c r="N28" s="5"/>
     </row>
     <row r="29" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="C29" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="F29" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
+        <v>70</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>93</v>
+      </c>
       <c r="K29" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L29" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="M29" s="7"/>
+      <c r="M29" s="7">
+        <v>45639</v>
+      </c>
       <c r="N29" s="5"/>
     </row>
     <row r="30" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="C30" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F30" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
+        <v>70</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>92</v>
+      </c>
       <c r="K30" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L30" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="M30" s="7"/>
+      <c r="M30" s="7">
+        <v>45639</v>
+      </c>
       <c r="N30" s="5"/>
     </row>
-    <row r="31" spans="1:14" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="C31" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="F31" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
+        <v>70</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>95</v>
+      </c>
       <c r="K31" s="6" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="L31" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="M31" s="7"/>
+      <c r="M31" s="7">
+        <v>45639</v>
+      </c>
       <c r="N31" s="5"/>
     </row>
-    <row r="32" spans="1:14" ht="87" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>